<commit_message>
Changes done accordingly #93
</commit_message>
<xml_diff>
--- a/Deliverable/Interface_Board/BOM/LCSC_BOM.xlsx
+++ b/Deliverable/Interface_Board/BOM/LCSC_BOM.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="440">
   <si>
     <t>Bill of Material (BOM) for Grant</t>
   </si>
@@ -1396,7 +1396,27 @@
     <t>Total Cost</t>
   </si>
   <si>
-    <t>R19, RF22, RF23</t>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>R18</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>,R19, RF22, RF23</t>
+    </r>
+  </si>
+  <si>
+    <t>DO NOT Mount R18</t>
   </si>
 </sst>
 </file>
@@ -1405,10 +1425,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000_);[Red]\(&quot;$&quot;#,##0.0000\)"/>
-    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="168" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
+    <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1562,6 +1582,24 @@
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -2113,7 +2151,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="180">
+  <cellXfs count="182">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2438,13 +2476,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="16" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="16" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2468,10 +2506,10 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="19" fillId="4" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="19" fillId="4" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="19" fillId="4" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="4" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2652,6 +2690,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5941,7 +5985,7 @@
       <c r="C39" s="124" t="s">
         <v>252</v>
       </c>
-      <c r="D39" s="125" t="s">
+      <c r="D39" s="180" t="s">
         <v>438</v>
       </c>
       <c r="E39" s="126" t="s">
@@ -6010,7 +6054,9 @@
         <f t="shared" si="17"/>
         <v>0.35</v>
       </c>
-      <c r="Y39" s="92"/>
+      <c r="Y39" s="181" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="40" spans="1:25">
       <c r="A40" s="7">
@@ -8865,7 +8911,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555602" right="0.30555555555555602" top="0.30555555555555602" bottom="0.30555555555555602" header="0" footer="0"/>
-  <pageSetup orientation="landscape" blackAndWhite="1"/>
+  <pageSetup orientation="landscape" blackAndWhite="1" r:id="rId67"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>